<commit_message>
descargar el driver del autentificador
</commit_message>
<xml_diff>
--- a/app/Plantillas.json/Entrada/eje3.xlsx
+++ b/app/Plantillas.json/Entrada/eje3.xlsx
@@ -753,13 +753,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEC68B-49C0-4864-8490-646DFCA76DD5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D786EBD5-71C6-4633-BB29-014C7AD95F8C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AF3D894-F1D8-4766-8D74-99129FF03985}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20FBAA6D-EC2A-4E3E-982E-2DB8CB978DA6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DC3C802-FFCA-4E2A-9FC0-A6DE4595461D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C9EE9AF-1532-4F11-8118-86D5D63FEF27}"/>
 </file>
</xml_diff>